<commit_message>
Carry the overlap case in the reference workbook
Intake_v1.xlsx now holds six records per 01 sheet: the full years 2021-2025
plus "2025 9 months". Two records therefore share the year 2025, so the
reference workbook exercises S10 directly instead of leaving it to tests
that construct the scenario in memory.

Both orientations carry the same six records and are still verified to
produce identical output. The partial period sits in a text-formatted cell
alongside numeric years, which also exercises the mixed-type key.

The control sum now counts 2025 twice, deliberately: with overlapping
periods it verifies extraction rather than being a portfolio total, and the
overlap hypothesis in the step-1 block says so.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgDs1kQm7zUEUCoe8K4YPd
</commit_message>
<xml_diff>
--- a/Intake_v1.xlsx
+++ b/Intake_v1.xlsx
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +140,7 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1142,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1396,50 +1397,76 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>2025 9 months</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>1180</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>7100</v>
+      </c>
+      <c r="L14" s="17">
+        <f>ROW()</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>H_PF transfer = with clean cut</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C14" s="18">
-        <f>SUM(C9:C13)</f>
-        <v>6910</v>
-      </c>
-      <c r="D14" s="18">
-        <f>SUM(D9:D13)</f>
-        <v>87750</v>
-      </c>
-      <c r="G14" s="18">
-        <f>SUM(G9:G13)</f>
-        <v>59570</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="C15" s="19">
+        <f>SUM(C9:C14)</f>
+        <v>8090</v>
+      </c>
+      <c r="D15" s="19">
+        <f>SUM(D9:D14)</f>
+        <v>102150</v>
+      </c>
+      <c r="G15" s="19">
+        <f>SUM(G9:G14)</f>
+        <v>66670</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>← selector empty: excluded from extraction, reused as control</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Info_1 = L</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>As at = 31.12.2025</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Note: 2025 figures preliminary</t>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Note: 2025 shown both as a full year and as the first nine months</t>
         </is>
       </c>
     </row>
@@ -1454,18 +1481,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1548,7 +1576,12 @@
       <c r="H8" s="13" t="n">
         <v>2025</v>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>2025 9 months</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1575,9 +1608,12 @@
       <c r="H9" s="14" t="n">
         <v>1505</v>
       </c>
-      <c r="I9" s="18">
-        <f>SUM(D9:H9)</f>
-        <v>6910</v>
+      <c r="I9" s="14" t="n">
+        <v>1180</v>
+      </c>
+      <c r="J9" s="19">
+        <f>SUM(D9:I9)</f>
+        <v>8090</v>
       </c>
     </row>
     <row r="10">
@@ -1611,9 +1647,12 @@
       <c r="H10" s="14" t="n">
         <v>19200</v>
       </c>
-      <c r="I10" s="18">
-        <f>SUM(D10:H10)</f>
-        <v>87750</v>
+      <c r="I10" s="14" t="n">
+        <v>14400</v>
+      </c>
+      <c r="J10" s="19">
+        <f>SUM(D10:I10)</f>
+        <v>102150</v>
       </c>
     </row>
     <row r="11">
@@ -1637,6 +1676,9 @@
       <c r="H11" s="15" t="n">
         <v>0.235</v>
       </c>
+      <c r="I11" s="15" t="n">
+        <v>0.235</v>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="7" t="inlineStr">
@@ -1659,6 +1701,9 @@
       <c r="H12" s="16" t="n">
         <v>1.05</v>
       </c>
+      <c r="I12" s="16" t="n">
+        <v>1.05</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1691,9 +1736,12 @@
       <c r="H13" s="14" t="n">
         <v>10250</v>
       </c>
-      <c r="I13" s="18">
-        <f>SUM(D13:H13)</f>
-        <v>59570</v>
+      <c r="I13" s="14" t="n">
+        <v>7100</v>
+      </c>
+      <c r="J13" s="19">
+        <f>SUM(D13:I13)</f>
+        <v>66670</v>
       </c>
     </row>
     <row r="16">
@@ -1727,6 +1775,10 @@
         <f>COLUMN()</f>
         <v>8</v>
       </c>
+      <c r="I16" s="17">
+        <f>COLUMN()</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
@@ -1738,7 +1790,7 @@
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Column I (Total) has no selector: excluded from extraction, reused as control.</t>
+          <t>The Total column has no selector: excluded from extraction, reused as control.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bring Intake_v1's sheet 00 up to the 04 specification
The Fire-only reference workbook still carried a greyed-out sketch of
dataset 04 with stale headers (Year, Event Date, Event Name, Incurred
Losses) and declared R-02 without its counterpart R-10. Sheet 00 is the
treaty's vocabulary, not an inventory of the sheets that happen to be in
one pack, so 04 is now declared in full there too — headers, the
'Occurrence year from' attribute and its vocabulary, the new field types,
and R-10. Both cat rules report 'not applicable' on a Fire pack, which is
structure rather than a gap.

Also: build_v1.py never injected the formula cache, so re-running it
produced a workbook whose =ROW() selectors had no cached value — fatal by
design, and only masked because the committed file had inject run out of
band. The script now does it itself and is reproducible.
</commit_message>
<xml_diff>
--- a/Intake_v1.xlsx
+++ b/Intake_v1.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:V88"/>
+  <dimension ref="B1:V93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -561,7 +561,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Rows 8-9 are provisional sketches, not yet specified.</t>
+          <t>Greyed rows are provisional sketches, not yet specified. 04 is specified, though this Fire-only pack carries no cat sheet.</t>
         </is>
       </c>
     </row>
@@ -794,57 +794,92 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>04. Cat Losses</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>04 Cat</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Event ID</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Loss amount</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Event Date</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Event Name</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Incurred Losses</t>
-        </is>
-      </c>
-      <c r="N8" s="7" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Event End Date</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Number of Claims (optional)</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
       </c>
-      <c r="P8" s="7" t="inlineStr">
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Share basis</t>
+        </is>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
         <is>
           <t>Year basis</t>
         </is>
       </c>
-      <c r="Q8" s="7" t="inlineStr">
+      <c r="S8" s="6" t="inlineStr">
         <is>
           <t>Loss basis</t>
         </is>
       </c>
-      <c r="R8" s="7" t="inlineStr">
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>Date format</t>
+        </is>
+      </c>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t>Occurrence year from</t>
+        </is>
+      </c>
+      <c r="V8" s="6" t="inlineStr">
         <is>
           <t>As at</t>
         </is>
@@ -1293,447 +1328,335 @@
     <row r="40">
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Loss amount</t>
+          <t>Event ID</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Date of Loss</t>
+          <t>Loss amount</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="4" t="inlineStr">
         <is>
+          <t>Number of Claims</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Date of Loss</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
           <t>Event Date</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="2" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Event End Date</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>A field name carries one type across the whole workbook. Year is text because 2026 and '2026 9 months' are two records.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>⟦VOCABULARY⟧</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="8" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>Permitted values</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Year basis</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>UW | Occurrence</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>Premium basis</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>GWP | GNPI | Written | Earned | Signed</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Loss basis</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Paid | Incurred</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>PF transfer</t>
+          <t>Year basis</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>with clean cut | without clean cut | none</t>
+          <t>UW | Occurrence</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Exposure basis</t>
+          <t>Premium basis</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Sum Insured | EML | PML | MPL</t>
+          <t>GWP | GNPI | Written | Earned | Signed</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Scale</t>
+          <t>Loss basis</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>1 | 1,000 | 1,000,000</t>
+          <t>Paid | Incurred</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Share basis</t>
+          <t>PF transfer</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>100% | ceded only</t>
+          <t>with clean cut | without clean cut | none</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Date format</t>
+          <t>Exposure basis</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>ISO | DD.MM.YYYY | MM/DD/YYYY</t>
+          <t>Sum Insured | EML | PML | MPL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="4" t="inlineStr">
         <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>1 | 1,000 | 1,000,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Share basis</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>100% | ceded only</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Date format</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>ISO | DD.MM.YYYY | MM/DD/YYYY</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Occurrence year from</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Event Date | Event End Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="4" t="inlineStr">
+        <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>ISO 4217</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="3" t="inlineStr">
+    <row r="63">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>⟦PERIOD ORDER⟧</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="8" t="inlineStr">
+    <row r="64">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="C60" s="8" t="inlineStr">
+      <c r="C64" s="8" t="inlineStr">
         <is>
           <t>Suffix</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="B61" s="10" t="n">
+    <row r="65">
+      <c r="B65" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="B62" s="10" t="n">
+    <row r="66">
+      <c r="B66" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>9 months</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="B63" s="10" t="n">
+    <row r="67">
+      <c r="B67" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>re-est</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="B65" s="2" t="inlineStr">
+    <row r="69">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>Within one year the suffixes sort in this order, not alphabetically: est comes before 9 months even though '9' &lt; 'e'. A bare year sorts first; an unlisted suffix sorts last.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="B67" s="3" t="inlineStr">
+    <row r="71">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>⟦RULES⟧</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>Left</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>Rel</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>Right</t>
-        </is>
-      </c>
-      <c r="F68" s="8" t="inlineStr">
-        <is>
-          <t>Tolerance</t>
-        </is>
-      </c>
-      <c r="G68" s="8" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="H68" s="8" t="inlineStr">
-        <is>
-          <t>Scope</t>
-        </is>
-      </c>
-      <c r="I68" s="8" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="8" t="inlineStr">
-        <is>
-          <t>R-05</t>
-        </is>
-      </c>
-      <c r="C69" s="11" t="inlineStr">
-        <is>
-          <t>01 History.Premium@{N} 9 months</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="E69" s="11" t="inlineStr">
-        <is>
-          <t>02 EPI.EPI@{N} 9 months</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="H69" s="5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>same nine months reported in two sheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>R-06</t>
-        </is>
-      </c>
-      <c r="C70" s="11" t="inlineStr">
-        <is>
-          <t>01 History.Premium@{N}</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="E70" s="11" t="inlineStr">
-        <is>
-          <t>02 EPI.EPI@{N} re-est</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="H70" s="5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>a full-year N in History is an estimate, not an actual</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="8" t="inlineStr">
-        <is>
-          <t>R-07</t>
-        </is>
-      </c>
-      <c r="C71" s="11" t="inlineStr">
-        <is>
-          <t>02 EPI.EPI@{N} re-est</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>&gt;=</t>
-        </is>
-      </c>
-      <c r="E71" s="11" t="inlineStr">
-        <is>
-          <t>02 EPI.EPI@{N} 9 months</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G71" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="H71" s="5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>premium accrues; a re-estimate cannot fall below what is booked</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>R-01</t>
-        </is>
-      </c>
-      <c r="C72" s="11" t="inlineStr">
-        <is>
-          <t>SUM(03 Large.Loss amount@{Y})</t>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>Left</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>&lt;=</t>
-        </is>
-      </c>
-      <c r="E72" s="11" t="inlineStr">
-        <is>
-          <t>01 History.Incurred Losses@{Y}</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G72" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>per risk</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>large losses cannot exceed total incurred for the same year</t>
+          <t>Rel</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>Tolerance</t>
+        </is>
+      </c>
+      <c r="G72" s="8" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="H72" s="8" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="I72" s="8" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>R-09</t>
+          <t>R-05</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>01 History.Year basis</t>
+          <t>01 History.Premium@{N} 9 months</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
@@ -1743,11 +1666,11 @@
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>03 Large.Year basis</t>
+          <t>02 EPI.EPI@{N} 9 months</t>
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
@@ -1756,34 +1679,34 @@
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>per risk</t>
+          <t>all</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>history and large losses must be on the same year basis</t>
+          <t>same nine months reported in two sheets</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>R-02</t>
+          <t>R-06</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>SUM(04 Cat.Loss amount@{Y})</t>
+          <t>01 History.Premium@{N}</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>&lt;=</t>
+          <t>=</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>01 History.Incurred Losses@{Y}</t>
+          <t>02 EPI.EPI@{N} re-est</t>
         </is>
       </c>
       <c r="F74" s="4" t="n">
@@ -1796,127 +1719,327 @@
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>a full-year N in History is an estimate, not an actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>R-07</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>02 EPI.EPI@{N} re-est</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>02 EPI.EPI@{N} 9 months</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>premium accrues; a re-estimate cannot fall below what is booked</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>R-01</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>SUM(03 Large.Loss amount@{Y})</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>01 History.Incurred Losses@{Y}</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>per risk</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>large losses cannot exceed total incurred for the same year</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>R-09</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>01 History.Year basis</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>03 Large.Year basis</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>per risk</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>history and large losses must be on the same year basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>R-02</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>SUM(04 Cat.Loss amount@{Y})</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>01 History.Incurred Losses@{Y}</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
           <t>cat</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
+      <c r="I78" s="2" t="inlineStr">
         <is>
           <t>cat losses cannot exceed total incurred for the same year</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>Forms: &lt;key&gt;.&lt;field&gt;@&lt;record&gt; · &lt;key&gt;.&lt;attribute&gt; · SUM(&lt;key&gt;.&lt;field&gt;@&lt;record&gt;).  {N} resolves from ⟦GLOBAL⟧; {Y} expands the rule once per year. A rule is skipped, not guessed, when a basis or currency differs; it is 'not applicable' when the dataset is absent from this pack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>⟦MARKERS⟧  —  written in column A of every other sheet</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="8" t="inlineStr">
         <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>01 History.Year basis</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>04 Cat.Year basis</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>cat</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>history and cat losses must be on the same year basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Forms: &lt;key&gt;.&lt;field&gt;@&lt;record&gt; · &lt;key&gt;.&lt;attribute&gt; · SUM(&lt;key&gt;.&lt;field&gt;@&lt;record&gt;).  {N} resolves from ⟦GLOBAL⟧; {Y} expands the rule once per year. A rule is skipped, not guessed, when a basis or currency differs; it is 'not applicable' when the dataset is absent from this pack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>⟦MARKERS⟧  —  written in column A of every other sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="8" t="inlineStr">
+        <is>
           <t>Marker</t>
         </is>
       </c>
-      <c r="C79" s="8" t="inlineStr">
+      <c r="C84" s="8" t="inlineStr">
         <is>
           <t>Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="B80" s="12" t="inlineStr">
-        <is>
-          <t>Header_i</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>row-wise: this row is block i's extraction row (declared labels only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="B81" s="12" t="inlineStr">
-        <is>
-          <t>Header_i = &lt;col&gt;</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>transposed: this column is block i's extraction column</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="B82" s="12" t="inlineStr">
-        <is>
-          <t>Info_i = &lt;col&gt;</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
-        <is>
-          <t>row-wise: this column holds the record selectors, =ROW()</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="12" t="inlineStr">
-        <is>
-          <t>Info_i = &lt;row&gt;</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>transposed: this row holds the record selectors, =COLUMN()</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" s="12" t="inlineStr">
-        <is>
-          <t>Transpose_i</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>block i is transposed</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t>&lt;Attribute&gt; = &lt;value&gt;</t>
+          <t>Header_i</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>an attribute of the sheet (unsuffixed) or block i (suffixed _i)</t>
+          <t>row-wise: this row is block i's extraction row (declared labels only)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" s="12" t="inlineStr">
         <is>
+          <t>Header_i = &lt;col&gt;</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>transposed: this column is block i's extraction column</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>Info_i = &lt;col&gt;</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>row-wise: this column holds the record selectors, =ROW()</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>Info_i = &lt;row&gt;</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>transposed: this row holds the record selectors, =COLUMN()</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>Transpose_i</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>block i is transposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>&lt;Attribute&gt; = &lt;value&gt;</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>an attribute of the sheet (unsuffixed) or block i (suffixed _i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="12" t="inlineStr">
+        <is>
           <t>H_&lt;Attribute&gt; = &lt;val&gt;</t>
         </is>
       </c>
-      <c r="C86" s="4" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>the same, declared as a hypothesis — raises a query</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="B88" s="8" t="inlineStr">
+    <row r="93">
+      <c r="B93" s="8" t="inlineStr">
         <is>
           <t>No Header_i anywhere in column A  →  nothing is extracted from that sheet.</t>
         </is>

</xml_diff>